<commit_message>
feat: implement unified field extraction service and add end-to-end ATC pipeline tests
</commit_message>
<xml_diff>
--- a/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
+++ b/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
@@ -17,13 +17,31 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002C3E50"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00145A32"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -44,14 +62,13 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00000000"/>
+      <color rgb="00566573"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -70,19 +87,31 @@
       <color rgb="007D6608"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="002C3E50"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6F7"/>
+        <bgColor rgb="00F4F6F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EFDF"/>
+        <bgColor rgb="00D4EFDF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -94,6 +123,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF0F2"/>
         <bgColor rgb="00FFF0F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F4F4"/>
+        <bgColor rgb="00F2F4F4"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,51 +182,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -559,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -570,666 +611,688 @@
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>TENDER EXTRACTION COMPLETENESS &amp; HEALTH SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total Schema Fields: 82  |  OK (Extracted): 43  |  OK (Fallback): 0  |  N/A (Not Applicable): 39  |  ⚠️ MISSING: 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>✅ COMPLETE — All expected fields successfully resolved with zero missing extractions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="12" customHeight="1"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
           <t>Organization:</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Sh. Boda Pool Singh</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Tender Name:</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>page6 177Tender 22ca0964 3fdd 4183 bbb81772690505617 buyer1.gil.rj</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Tender ID:</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>GEM/2026/B/7306631 (Ref No.: GAIL/C&amp;P/JPR25BP177/2025-26)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Website:</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>is negative / black</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Bid Due Date and Time</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>specified</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Recommendation by TE</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>of the fact that any</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Tender Information</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Processing Fees</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Processing Fees (in form of)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Tender Fees</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Tender Fees (in form of)</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>EMD</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>₹1,94,177</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>EMD required</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Tender Value (GST Inclusive)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>EMD (in form of)</t>
         </is>
       </c>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>BT/DD/SB/FDR/BG</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Bid Validity</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>16 Days</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Commercial Evaluation</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Techno-commercially acceptable/ responsive bids shall be evaluated and</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>RA Applicable</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Bid Type</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>SINGLE BID  SYSTEM</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>ATC Document Link</t>
         </is>
       </c>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>MAF required</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Delivery Time (Supply/Total)</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>3 months</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>Delivery Time (Installation)</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Inclusive (SITC Scope)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>PBG (in form of)</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>DD / Online Transfer / Insurance Surety Bond / FDR / Bank Guarantee</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Payment Terms (Supply)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Payment Terms (Installation)</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>SD (in form of)</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Bank Guarantee / DD / FDR / Online Transfer / Insurance Surety Bond</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>LD/PRS %age (per week)</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Max LD %age</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>PBG Required</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>PBG %age</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Security Deposit</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>PBG Duration</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>SD Duration</t>
         </is>
       </c>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Physical Docs Submission Required</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Physical Docs Submission Deadline</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Within 7 (seven) days</t>
         </is>
       </c>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="F24" s="12" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Eligibility Criterion</t>
         </is>
       </c>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>Age (in yrs)</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Financial Criterion</t>
         </is>
       </c>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>3 Works Value</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Annual Avg Turnover</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>₹0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>2 Works Value</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>₹0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>1 work Value</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Net Worth</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>₹0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>PO selected for Technical Eligibility</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Solvency Certificate</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>₹0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="55" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>PQC Documents</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Document-1, Document-2, Document-3 (Auto attach the documents from PQR dashboard, based on the name selection)</t>
         </is>
       </c>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Documents for Commercial Eligibility</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Custom Eligibility Criteria</t>
         </is>
       </c>
-      <c r="B28" s="1" t="n"/>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Minimum Qualifying Order Value: Rs. 62.14 Lakhs (6214000 INR)</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="10" customHeight="1">
-      <c r="A29" s="9" t="inlineStr"/>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+    </row>
+    <row r="33" ht="10" customHeight="1">
+      <c r="A33" s="12" t="inlineStr"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Client Name</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Sh. Boda Pool Singh</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>poolsingh.boda@gail.co.in</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>0141-2230347/617/698 (Extn. 860-
 1385). 
@@ -1237,475 +1300,479 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Client Name</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>. The Fraud Prevention Policy document i</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Shri Sheew Shankar</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>sheewshankar@gail.co.in</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>0141-2230347 
+E</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Client Name</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="10" customHeight="1">
-      <c r="A33" s="9" t="inlineStr"/>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="10" customHeight="1">
+      <c r="A37" s="12" t="inlineStr"/>
+      <c r="B37" s="12" t="n"/>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="12" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="12" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Documents Submitted</t>
         </is>
       </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Doc 1</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>To:</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>Doc 2</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Doc 3</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Doc 4</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>Doc 5</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>Doc 6</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Doc 7</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>Doc 8</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Doc 9</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Courier Delivery Address</t>
         </is>
       </c>
-      <c r="B38" s="9" t="n"/>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>GAIL (India) Limited, GAIL Bhawan, Sector-6, Vidhyadhar Nagar, Jaipur, Rajasthan– 302039. | Kind Attn: Sh. Boda Pool Singh (poolsingh.boda@gail.co.in)</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
-      <c r="F38" s="9" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Courier Provider</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>Courier Docket No.</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Delivery time</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Docket slip - Upload</t>
         </is>
       </c>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>Physical Documents Couriered - Upload</t>
         </is>
       </c>
-      <c r="E40" s="9" t="n"/>
-      <c r="F40" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="10" customHeight="1">
-      <c r="A41" s="9" t="inlineStr"/>
-      <c r="B41" s="9" t="n"/>
-      <c r="C41" s="9" t="n"/>
-      <c r="D41" s="9" t="n"/>
-      <c r="E41" s="9" t="n"/>
-      <c r="F41" s="9" t="n"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="10" customHeight="1">
+      <c r="A45" s="12" t="inlineStr"/>
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>Evaluation &amp; Preference Policies</t>
         </is>
       </c>
-      <c r="B42" s="8" t="n"/>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
-      <c r="E42" s="8" t="n"/>
-      <c r="F42" s="8" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>MSE Relaxation</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n"/>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="B47" s="12" t="n"/>
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Exempt / Not Applicable</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>Startup Relaxation</t>
         </is>
       </c>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="12" t="inlineStr">
         <is>
           <t>Exempt / Not Applicable</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="9" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>MSE Purchase Preference</t>
         </is>
       </c>
-      <c r="B44" s="9" t="n"/>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="B48" s="12" t="n"/>
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>MII Purchase Preference</t>
         </is>
       </c>
-      <c r="E44" s="9" t="n"/>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Pre-Bid Meeting Details</t>
         </is>
       </c>
-      <c r="B45" s="9" t="n"/>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>Through VC via Microsoft Teams meeting.</t>
         </is>
       </c>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9" t="n"/>
-    </row>
-    <row r="46" ht="10" customHeight="1">
-      <c r="A46" s="9" t="inlineStr"/>
-      <c r="B46" s="9" t="n"/>
-      <c r="C46" s="9" t="n"/>
-      <c r="D46" s="9" t="n"/>
-      <c r="E46" s="9" t="n"/>
-      <c r="F46" s="9" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+    </row>
+    <row r="50" ht="10" customHeight="1">
+      <c r="A50" s="12" t="inlineStr"/>
+      <c r="B50" s="12" t="n"/>
+      <c r="C50" s="12" t="n"/>
+      <c r="D50" s="12" t="n"/>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="12" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Schedule &amp; Technical Specifications</t>
         </is>
       </c>
-      <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="n"/>
-      <c r="D47" s="8" t="n"/>
-      <c r="E47" s="8" t="n"/>
-      <c r="F47" s="8" t="n"/>
-    </row>
-    <row r="48" ht="40" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="11" t="n"/>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>Schedule 1 Details</t>
         </is>
       </c>
-      <c r="B48" s="9" t="n"/>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>Sch 1 | Qty: 7 | Delivery: Not Found days | Government/ Organizations in previous seven (07) | Specs: MSEs) or otherwise] subject to their meeting the quality and technical specifications specified: in tender document., 10. The Guarantor represents and confirms that the Guarantor has the legal capacity, power and: authority to issue this Guarantee and that giving of this Guarantee and the performance and, h). Complaints against specifications except under the premise that they are either vague or: vendor/ contractor; and, their meeting the quality and technical specifications specified in tender document and: submission of document specified in Section-II., specifications including all addenda/corrigenda published before entering into the Contract, as: applicable and specified in the Contract., iii) Specific Technical Specification/Job Specifications (pertaining to Scope of Supply): (iv) Drawings, vi) General Technical Specifications (if applicable): SV Stations with Buy Back” under GAIL Abu Road., Specifications or drawings, but which are usual or necessary for the satisfactory functioning of: the Goods ( i.e. successful operation and functioning of the Equipment being Supplier’s, the quantities, specifications, drawings etc. without changing the indented purpose of the: Contract. If such changes cause an increase or decrease in the price or time required for the, and/or the Technical Specifications shall specify what inspections and tests the Purchaser: requires and where they are to be conducted. The Purchaser shall notify the Supplier in writing, found not conforming to the requirements/specifications of the Purchase Order, shall be liable: for immediate rejection. Supplier shall be responsible and liable for immediate replacement of, No deviation from such specifications or alterations or of these conditions shall be made without: Purchaser’s /Consultant’s agreement in writing which must be obtained before any work against, In the event that the materials supplied do not meet the specifications and/or not in accordance: with the drawings data sheets or the terms of the Contract (including guarantee period) and, standards, the job specification contained herein &amp; codes referred to. Where the job: specifications stipulate requirements in additions to those contained in the standard codes and, reports for approval. All acceptance and routine tests as per the specification and relevant: SV Stations with Buy Back” under GAIL Abu Road.</t>
         </is>
       </c>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
-      <c r="F48" s="9" t="n"/>
-    </row>
-    <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="9" t="inlineStr">
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Schedule 2 Details</t>
         </is>
       </c>
-      <c r="B49" s="9" t="n"/>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="B53" s="12" t="n"/>
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>Sch 2 | Qty: 7 | Delivery: Not Found days | within previous seven (07) | Specs: specifications and to fulfil the foregoing guarantees. However, in no case, warranty of: repaired/replaced part shall exceed 24 months from the date of commissioning of original, 4.01 All standards, specifications and codes of practice referred to herein, shall be the latest editions: including all applicable official amendments and revisions as on date of opening of techno, In case of conflict between this specification and those (IS codes, Standards etc.) referred to herein,: the former shall prevail. All works shall be carried out as per the following standards and codes:</t>
         </is>
       </c>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
-      <c r="F49" s="9" t="n"/>
-    </row>
-    <row r="50" ht="40" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
+      <c r="D53" s="12" t="n"/>
+      <c r="E53" s="12" t="n"/>
+      <c r="F53" s="12" t="n"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>Schedule 3 Details</t>
         </is>
       </c>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="B54" s="12" t="n"/>
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>Sch 3 | Qty: 4 | Delivery: Not Found days | 5. "Beneficial owner" for the purpose of above (4) | Specs:  ⚠ QTY MISMATCH: schedules sum 18.0 vs header total 51025.0</t>
         </is>
       </c>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="9" t="n"/>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12" t="n"/>
+      <c r="F54" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="63">
-    <mergeCell ref="A41:F41"/>
+  <mergeCells count="66">
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C52:F52"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A46:F46"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="D21:F21"/>
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A33:F33"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C49:F49"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="C6:F6"/>
     <mergeCell ref="C5:F5"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C42:F42"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="A47:B47"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D9:E9"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C17:D17"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="D23:E23"/>
     <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D14:E14"/>
     <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A40:B40"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="D6:F6"/>
     <mergeCell ref="D44:E44"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement tender ingestion pipeline with field mapping, alias definitions, and workspace integration
</commit_message>
<xml_diff>
--- a/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
+++ b/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
@@ -621,7 +621,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Schema Fields: 82  |  OK (Extracted): 43  |  OK (Fallback): 0  |  N/A (Not Applicable): 39  |  ⚠️ MISSING: 0</t>
+          <t>Total Schema Fields: 82  |  OK (Extracted): 41  |  OK (Fallback): 0  |  N/A (Not Applicable): 41  |  ⚠️ MISSING: 0</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Sh. Boda Pool Singh</t>
+          <t>Boda Pool Singh, Sr. Officer (C&amp;P)</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -1282,9 +1282,9 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>poolsingh.boda@gail.co.in</t>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -1292,11 +1292,9 @@
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>0141-2230347/617/698 (Extn. 860-
-1385). 
-E-</t>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1488,7 @@
       <c r="B42" s="12" t="n"/>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>GAIL (India) Limited, GAIL Bhawan, Sector-6, Vidhyadhar Nagar, Jaipur, Rajasthan– 302039. | Kind Attn: Sh. Boda Pool Singh (poolsingh.boda@gail.co.in)</t>
+          <t>GAIL (India) Limited,</t>
         </is>
       </c>
       <c r="D42" s="12" t="n"/>

</xml_diff>

<commit_message>
feat: implement LLM-based field resolver for GAIL/GeM ATC parsing with few-shot memory and schema-typed extraction.
</commit_message>
<xml_diff>
--- a/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
+++ b/sample_files/extracted_children/page6_177Tender_22ca0964-3fdd-4183-bbb81772690505617_buyer1.gil.rj_InfoSheet.xlsx
@@ -929,7 +929,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Inclusive (SITC Scope)</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>

</xml_diff>